<commit_message>
Updated simple Obs and DiagRep
</commit_message>
<xml_diff>
--- a/314e-ig/output/StructureDefinition-diagnosticreport-314e.xlsx
+++ b/314e-ig/output/StructureDefinition-diagnosticreport-314e.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1781" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1852" uniqueCount="447">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-18T14:15:04+05:30</t>
+    <t>2026-06-18T16:14:31+05:30</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -608,10 +608,12 @@
 </t>
   </si>
   <si>
-    <t>Service category</t>
-  </si>
-  <si>
-    <t>A code that classifies the clinical discipline, department or diagnostic service that created the report (e.g. cardiology, biochemistry, hematology, MRI). This is used for searching, sorting and display purposes.</t>
+    <t>Operational procedure/service categories</t>
+  </si>
+  <si>
+    <t>Broad and optional subcategory classifications used
+for workflow, routing, analytics, and operational
+grouping of DiagnosticReport resources.</t>
   </si>
   <si>
     <t>Multiple categories are allowed using various categorization schemes.   The level of granularity is defined by the category concepts in the value set. More fine-grained filtering can be performed using the metadata and/or terminology hierarchy in DiagnosticReport.code.</t>
@@ -626,6 +628,10 @@
     <t>http://hl7.org/fhir/ValueSet/diagnostic-service-sections|4.0.1</t>
   </si>
   <si>
+    <t xml:space="preserve">pattern:$this}
+</t>
+  </si>
+  <si>
     <t>OBR-24</t>
   </si>
   <si>
@@ -633,6 +639,38 @@
   </si>
   <si>
     <t>FiveWs.class</t>
+  </si>
+  <si>
+    <t>DiagnosticReport.category:broadCategory</t>
+  </si>
+  <si>
+    <t>broadCategory</t>
+  </si>
+  <si>
+    <t>Required broad procedure/service category</t>
+  </si>
+  <si>
+    <t>Top-level operational classification of the
+diagnostic report.</t>
+  </si>
+  <si>
+    <t>http://314e.com/fhir/ValueSet/procedure-category-broad-314e</t>
+  </si>
+  <si>
+    <t>DiagnosticReport.category:subCategory</t>
+  </si>
+  <si>
+    <t>subCategory</t>
+  </si>
+  <si>
+    <t>Optional detailed subcategory</t>
+  </si>
+  <si>
+    <t>More granular operational sub-classification of the
+diagnostic report.</t>
+  </si>
+  <si>
+    <t>http://314e.com/fhir/ValueSet/procedure-category-subcategory-314e</t>
   </si>
   <si>
     <t>DiagnosticReport.code</t>
@@ -1692,12 +1730,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AN48"/>
+  <dimension ref="A1:AN50"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="49.46484375" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="38.25390625" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="12.16796875" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="3" max="3" width="12.8671875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="54.296875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.29296875" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="4.21484375" customWidth="true" bestFit="true"/>
@@ -1720,7 +1758,7 @@
     <col min="23" max="23" width="15.31640625" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="14.62890625" customWidth="true" bestFit="true"/>
     <col min="25" max="25" width="53.48828125" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="50.59765625" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="57.36328125" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.10546875" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="17.6953125" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="35.90625" customWidth="true" bestFit="true"/>
@@ -3353,7 +3391,7 @@
       </c>
       <c r="E15" s="2"/>
       <c r="F15" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="G15" t="s" s="2">
         <v>79</v>
@@ -3415,16 +3453,14 @@
         <v>20</v>
       </c>
       <c r="AB15" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AC15" t="s" s="2">
-        <v>20</v>
-      </c>
+        <v>194</v>
+      </c>
+      <c r="AC15" s="2"/>
       <c r="AD15" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AE15" t="s" s="2">
-        <v>20</v>
+        <v>138</v>
       </c>
       <c r="AF15" t="s" s="2">
         <v>185</v>
@@ -3445,25 +3481,27 @@
         <v>20</v>
       </c>
       <c r="AL15" t="s" s="2">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AM15" t="s" s="2">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="AN15" t="s" s="2">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>197</v>
-      </c>
-      <c r="C16" s="2"/>
+        <v>185</v>
+      </c>
+      <c r="C16" t="s" s="2">
+        <v>199</v>
+      </c>
       <c r="D16" t="s" s="2">
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="E16" s="2"/>
       <c r="F16" t="s" s="2">
@@ -3485,12 +3523,14 @@
         <v>187</v>
       </c>
       <c r="L16" t="s" s="2">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="M16" t="s" s="2">
-        <v>200</v>
-      </c>
-      <c r="N16" s="2"/>
+        <v>201</v>
+      </c>
+      <c r="N16" t="s" s="2">
+        <v>190</v>
+      </c>
       <c r="O16" s="2"/>
       <c r="P16" t="s" s="2">
         <v>20</v>
@@ -3515,11 +3555,9 @@
         <v>20</v>
       </c>
       <c r="X16" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="Y16" t="s" s="2">
-        <v>201</v>
-      </c>
+        <v>179</v>
+      </c>
+      <c r="Y16" s="2"/>
       <c r="Z16" t="s" s="2">
         <v>202</v>
       </c>
@@ -3539,13 +3577,13 @@
         <v>20</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>197</v>
+        <v>185</v>
       </c>
       <c r="AG16" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="AH16" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="AI16" t="s" s="2">
         <v>20</v>
@@ -3554,28 +3592,30 @@
         <v>101</v>
       </c>
       <c r="AK16" t="s" s="2">
-        <v>203</v>
+        <v>20</v>
       </c>
       <c r="AL16" t="s" s="2">
-        <v>204</v>
+        <v>195</v>
       </c>
       <c r="AM16" t="s" s="2">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="AN16" t="s" s="2">
-        <v>206</v>
+        <v>197</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>207</v>
-      </c>
-      <c r="C17" s="2"/>
+        <v>185</v>
+      </c>
+      <c r="C17" t="s" s="2">
+        <v>204</v>
+      </c>
       <c r="D17" t="s" s="2">
-        <v>208</v>
+        <v>186</v>
       </c>
       <c r="E17" s="2"/>
       <c r="F17" t="s" s="2">
@@ -3594,18 +3634,18 @@
         <v>90</v>
       </c>
       <c r="K17" t="s" s="2">
-        <v>209</v>
+        <v>187</v>
       </c>
       <c r="L17" t="s" s="2">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>211</v>
-      </c>
-      <c r="N17" s="2"/>
-      <c r="O17" t="s" s="2">
-        <v>212</v>
-      </c>
+        <v>206</v>
+      </c>
+      <c r="N17" t="s" s="2">
+        <v>190</v>
+      </c>
+      <c r="O17" s="2"/>
       <c r="P17" t="s" s="2">
         <v>20</v>
       </c>
@@ -3629,13 +3669,11 @@
         <v>20</v>
       </c>
       <c r="X17" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="Y17" t="s" s="2">
-        <v>20</v>
-      </c>
+        <v>179</v>
+      </c>
+      <c r="Y17" s="2"/>
       <c r="Z17" t="s" s="2">
-        <v>20</v>
+        <v>207</v>
       </c>
       <c r="AA17" t="s" s="2">
         <v>20</v>
@@ -3653,13 +3691,13 @@
         <v>20</v>
       </c>
       <c r="AF17" t="s" s="2">
-        <v>207</v>
+        <v>185</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH17" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="AI17" t="s" s="2">
         <v>20</v>
@@ -3668,32 +3706,32 @@
         <v>101</v>
       </c>
       <c r="AK17" t="s" s="2">
-        <v>213</v>
+        <v>20</v>
       </c>
       <c r="AL17" t="s" s="2">
-        <v>214</v>
+        <v>195</v>
       </c>
       <c r="AM17" t="s" s="2">
-        <v>215</v>
+        <v>196</v>
       </c>
       <c r="AN17" t="s" s="2">
-        <v>216</v>
+        <v>197</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="G18" t="s" s="2">
         <v>89</v>
@@ -3708,20 +3746,16 @@
         <v>90</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>219</v>
+        <v>187</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>221</v>
-      </c>
-      <c r="N18" t="s" s="2">
-        <v>222</v>
-      </c>
-      <c r="O18" t="s" s="2">
-        <v>223</v>
-      </c>
+        <v>211</v>
+      </c>
+      <c r="N18" s="2"/>
+      <c r="O18" s="2"/>
       <c r="P18" t="s" s="2">
         <v>20</v>
       </c>
@@ -3745,13 +3779,13 @@
         <v>20</v>
       </c>
       <c r="X18" t="s" s="2">
-        <v>20</v>
+        <v>113</v>
       </c>
       <c r="Y18" t="s" s="2">
-        <v>20</v>
+        <v>212</v>
       </c>
       <c r="Z18" t="s" s="2">
-        <v>20</v>
+        <v>213</v>
       </c>
       <c r="AA18" t="s" s="2">
         <v>20</v>
@@ -3769,10 +3803,10 @@
         <v>20</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="AG18" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="AH18" t="s" s="2">
         <v>89</v>
@@ -3784,28 +3818,28 @@
         <v>101</v>
       </c>
       <c r="AK18" t="s" s="2">
-        <v>224</v>
+        <v>214</v>
       </c>
       <c r="AL18" t="s" s="2">
-        <v>225</v>
+        <v>215</v>
       </c>
       <c r="AM18" t="s" s="2">
-        <v>226</v>
+        <v>216</v>
       </c>
       <c r="AN18" t="s" s="2">
-        <v>227</v>
+        <v>217</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>228</v>
+        <v>218</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>228</v>
+        <v>218</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
-        <v>229</v>
+        <v>219</v>
       </c>
       <c r="E19" s="2"/>
       <c r="F19" t="s" s="2">
@@ -3824,19 +3858,17 @@
         <v>90</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>230</v>
+        <v>220</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>232</v>
-      </c>
-      <c r="N19" t="s" s="2">
-        <v>233</v>
-      </c>
+        <v>222</v>
+      </c>
+      <c r="N19" s="2"/>
       <c r="O19" t="s" s="2">
-        <v>234</v>
+        <v>223</v>
       </c>
       <c r="P19" t="s" s="2">
         <v>20</v>
@@ -3885,7 +3917,7 @@
         <v>20</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>228</v>
+        <v>218</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>78</v>
@@ -3900,28 +3932,28 @@
         <v>101</v>
       </c>
       <c r="AK19" t="s" s="2">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="AL19" t="s" s="2">
-        <v>236</v>
+        <v>225</v>
       </c>
       <c r="AM19" t="s" s="2">
-        <v>237</v>
+        <v>226</v>
       </c>
       <c r="AN19" t="s" s="2">
-        <v>238</v>
+        <v>227</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
-        <v>240</v>
+        <v>229</v>
       </c>
       <c r="E20" s="2"/>
       <c r="F20" t="s" s="2">
@@ -3940,19 +3972,19 @@
         <v>90</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>241</v>
+        <v>230</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>242</v>
+        <v>231</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>243</v>
+        <v>232</v>
       </c>
       <c r="N20" t="s" s="2">
-        <v>244</v>
+        <v>233</v>
       </c>
       <c r="O20" t="s" s="2">
-        <v>245</v>
+        <v>234</v>
       </c>
       <c r="P20" t="s" s="2">
         <v>20</v>
@@ -4001,7 +4033,7 @@
         <v>20</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>78</v>
@@ -4016,35 +4048,35 @@
         <v>101</v>
       </c>
       <c r="AK20" t="s" s="2">
-        <v>20</v>
+        <v>235</v>
       </c>
       <c r="AL20" t="s" s="2">
-        <v>246</v>
+        <v>236</v>
       </c>
       <c r="AM20" t="s" s="2">
-        <v>247</v>
+        <v>237</v>
       </c>
       <c r="AN20" t="s" s="2">
-        <v>248</v>
+        <v>238</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>249</v>
+        <v>239</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>249</v>
+        <v>239</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="E21" s="2"/>
       <c r="F21" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G21" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="H21" t="s" s="2">
         <v>20</v>
@@ -4056,19 +4088,19 @@
         <v>90</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>252</v>
+        <v>242</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>253</v>
+        <v>243</v>
       </c>
       <c r="N21" t="s" s="2">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="O21" t="s" s="2">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="P21" t="s" s="2">
         <v>20</v>
@@ -4117,13 +4149,13 @@
         <v>20</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>249</v>
+        <v>239</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH21" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="AI21" t="s" s="2">
         <v>20</v>
@@ -4132,35 +4164,35 @@
         <v>101</v>
       </c>
       <c r="AK21" t="s" s="2">
-        <v>256</v>
+        <v>246</v>
       </c>
       <c r="AL21" t="s" s="2">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="AM21" t="s" s="2">
-        <v>258</v>
+        <v>248</v>
       </c>
       <c r="AN21" t="s" s="2">
-        <v>259</v>
+        <v>249</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
-        <v>261</v>
+        <v>251</v>
       </c>
       <c r="E22" s="2"/>
       <c r="F22" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G22" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="H22" t="s" s="2">
         <v>20</v>
@@ -4172,19 +4204,19 @@
         <v>90</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>262</v>
+        <v>253</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>263</v>
+        <v>254</v>
       </c>
       <c r="N22" t="s" s="2">
-        <v>264</v>
+        <v>255</v>
       </c>
       <c r="O22" t="s" s="2">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="P22" t="s" s="2">
         <v>20</v>
@@ -4233,13 +4265,13 @@
         <v>20</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH22" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="AI22" t="s" s="2">
         <v>20</v>
@@ -4248,10 +4280,10 @@
         <v>101</v>
       </c>
       <c r="AK22" t="s" s="2">
-        <v>256</v>
+        <v>20</v>
       </c>
       <c r="AL22" t="s" s="2">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="AM22" t="s" s="2">
         <v>258</v>
@@ -4262,14 +4294,14 @@
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
-        <v>20</v>
+        <v>261</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" t="s" s="2">
@@ -4285,22 +4317,22 @@
         <v>20</v>
       </c>
       <c r="J23" t="s" s="2">
-        <v>20</v>
+        <v>90</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="N23" t="s" s="2">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="O23" t="s" s="2">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="P23" t="s" s="2">
         <v>20</v>
@@ -4349,7 +4381,7 @@
         <v>20</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>78</v>
@@ -4364,28 +4396,28 @@
         <v>101</v>
       </c>
       <c r="AK23" t="s" s="2">
-        <v>20</v>
+        <v>267</v>
       </c>
       <c r="AL23" t="s" s="2">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="AM23" t="s" s="2">
-        <v>215</v>
+        <v>269</v>
       </c>
       <c r="AN23" t="s" s="2">
-        <v>20</v>
+        <v>270</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="E24" s="2"/>
       <c r="F24" t="s" s="2">
@@ -4401,22 +4433,22 @@
         <v>20</v>
       </c>
       <c r="J24" t="s" s="2">
-        <v>20</v>
+        <v>90</v>
       </c>
       <c r="K24" t="s" s="2">
+        <v>262</v>
+      </c>
+      <c r="L24" t="s" s="2">
+        <v>273</v>
+      </c>
+      <c r="M24" t="s" s="2">
+        <v>274</v>
+      </c>
+      <c r="N24" t="s" s="2">
         <v>275</v>
       </c>
-      <c r="L24" t="s" s="2">
-        <v>276</v>
-      </c>
-      <c r="M24" t="s" s="2">
-        <v>277</v>
-      </c>
-      <c r="N24" t="s" s="2">
-        <v>278</v>
-      </c>
       <c r="O24" t="s" s="2">
-        <v>279</v>
+        <v>266</v>
       </c>
       <c r="P24" t="s" s="2">
         <v>20</v>
@@ -4465,7 +4497,7 @@
         <v>20</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>78</v>
@@ -4480,24 +4512,24 @@
         <v>101</v>
       </c>
       <c r="AK24" t="s" s="2">
-        <v>20</v>
+        <v>267</v>
       </c>
       <c r="AL24" t="s" s="2">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="AM24" t="s" s="2">
-        <v>281</v>
+        <v>269</v>
       </c>
       <c r="AN24" t="s" s="2">
-        <v>20</v>
+        <v>270</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -4520,18 +4552,20 @@
         <v>20</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="N25" t="s" s="2">
-        <v>286</v>
-      </c>
-      <c r="O25" s="2"/>
+        <v>281</v>
+      </c>
+      <c r="O25" t="s" s="2">
+        <v>282</v>
+      </c>
       <c r="P25" t="s" s="2">
         <v>20</v>
       </c>
@@ -4579,7 +4613,7 @@
         <v>20</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>78</v>
@@ -4597,10 +4631,10 @@
         <v>20</v>
       </c>
       <c r="AL25" t="s" s="2">
-        <v>20</v>
+        <v>283</v>
       </c>
       <c r="AM25" t="s" s="2">
-        <v>287</v>
+        <v>226</v>
       </c>
       <c r="AN25" t="s" s="2">
         <v>20</v>
@@ -4608,14 +4642,14 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="E26" s="2"/>
       <c r="F26" t="s" s="2">
@@ -4631,20 +4665,22 @@
         <v>20</v>
       </c>
       <c r="J26" t="s" s="2">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="K26" t="s" s="2">
+        <v>286</v>
+      </c>
+      <c r="L26" t="s" s="2">
+        <v>287</v>
+      </c>
+      <c r="M26" t="s" s="2">
+        <v>288</v>
+      </c>
+      <c r="N26" t="s" s="2">
+        <v>289</v>
+      </c>
+      <c r="O26" t="s" s="2">
         <v>290</v>
-      </c>
-      <c r="L26" t="s" s="2">
-        <v>291</v>
-      </c>
-      <c r="M26" t="s" s="2">
-        <v>292</v>
-      </c>
-      <c r="N26" s="2"/>
-      <c r="O26" t="s" s="2">
-        <v>293</v>
       </c>
       <c r="P26" t="s" s="2">
         <v>20</v>
@@ -4693,7 +4729,7 @@
         <v>20</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>78</v>
@@ -4711,10 +4747,10 @@
         <v>20</v>
       </c>
       <c r="AL26" t="s" s="2">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="AM26" t="s" s="2">
-        <v>281</v>
+        <v>292</v>
       </c>
       <c r="AN26" t="s" s="2">
         <v>20</v>
@@ -4722,10 +4758,10 @@
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -4736,7 +4772,7 @@
         <v>78</v>
       </c>
       <c r="G27" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="H27" t="s" s="2">
         <v>20</v>
@@ -4748,15 +4784,17 @@
         <v>20</v>
       </c>
       <c r="K27" t="s" s="2">
+        <v>294</v>
+      </c>
+      <c r="L27" t="s" s="2">
+        <v>295</v>
+      </c>
+      <c r="M27" t="s" s="2">
         <v>296</v>
       </c>
-      <c r="L27" t="s" s="2">
+      <c r="N27" t="s" s="2">
         <v>297</v>
       </c>
-      <c r="M27" t="s" s="2">
-        <v>298</v>
-      </c>
-      <c r="N27" s="2"/>
       <c r="O27" s="2"/>
       <c r="P27" t="s" s="2">
         <v>20</v>
@@ -4805,19 +4843,19 @@
         <v>20</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>299</v>
+        <v>293</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH27" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="AI27" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AJ27" t="s" s="2">
-        <v>20</v>
+        <v>101</v>
       </c>
       <c r="AK27" t="s" s="2">
         <v>20</v>
@@ -4826,7 +4864,7 @@
         <v>20</v>
       </c>
       <c r="AM27" t="s" s="2">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="AN27" t="s" s="2">
         <v>20</v>
@@ -4834,14 +4872,14 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
-        <v>148</v>
+        <v>300</v>
       </c>
       <c r="E28" s="2"/>
       <c r="F28" t="s" s="2">
@@ -4857,10 +4895,10 @@
         <v>20</v>
       </c>
       <c r="J28" t="s" s="2">
-        <v>20</v>
+        <v>90</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>134</v>
+        <v>301</v>
       </c>
       <c r="L28" t="s" s="2">
         <v>302</v>
@@ -4868,10 +4906,10 @@
       <c r="M28" t="s" s="2">
         <v>303</v>
       </c>
-      <c r="N28" t="s" s="2">
-        <v>151</v>
-      </c>
-      <c r="O28" s="2"/>
+      <c r="N28" s="2"/>
+      <c r="O28" t="s" s="2">
+        <v>304</v>
+      </c>
       <c r="P28" t="s" s="2">
         <v>20</v>
       </c>
@@ -4919,7 +4957,7 @@
         <v>20</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>78</v>
@@ -4931,16 +4969,16 @@
         <v>20</v>
       </c>
       <c r="AJ28" t="s" s="2">
-        <v>140</v>
+        <v>101</v>
       </c>
       <c r="AK28" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL28" t="s" s="2">
-        <v>20</v>
+        <v>305</v>
       </c>
       <c r="AM28" t="s" s="2">
-        <v>300</v>
+        <v>292</v>
       </c>
       <c r="AN28" t="s" s="2">
         <v>20</v>
@@ -4948,46 +4986,42 @@
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
-        <v>306</v>
+        <v>20</v>
       </c>
       <c r="E29" s="2"/>
       <c r="F29" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G29" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="H29" t="s" s="2">
         <v>20</v>
       </c>
       <c r="I29" t="s" s="2">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="J29" t="s" s="2">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>134</v>
+        <v>307</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>308</v>
-      </c>
-      <c r="N29" t="s" s="2">
-        <v>151</v>
-      </c>
-      <c r="O29" t="s" s="2">
-        <v>152</v>
-      </c>
+        <v>309</v>
+      </c>
+      <c r="N29" s="2"/>
+      <c r="O29" s="2"/>
       <c r="P29" t="s" s="2">
         <v>20</v>
       </c>
@@ -5035,19 +5069,19 @@
         <v>20</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH29" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="AI29" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AJ29" t="s" s="2">
-        <v>140</v>
+        <v>20</v>
       </c>
       <c r="AK29" t="s" s="2">
         <v>20</v>
@@ -5056,7 +5090,7 @@
         <v>20</v>
       </c>
       <c r="AM29" t="s" s="2">
-        <v>132</v>
+        <v>311</v>
       </c>
       <c r="AN29" t="s" s="2">
         <v>20</v>
@@ -5064,21 +5098,21 @@
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
-        <v>20</v>
+        <v>148</v>
       </c>
       <c r="E30" s="2"/>
       <c r="F30" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G30" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="H30" t="s" s="2">
         <v>20</v>
@@ -5090,20 +5124,18 @@
         <v>20</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>296</v>
+        <v>134</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="N30" t="s" s="2">
-        <v>313</v>
-      </c>
-      <c r="O30" t="s" s="2">
-        <v>314</v>
-      </c>
+        <v>151</v>
+      </c>
+      <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
         <v>20</v>
       </c>
@@ -5151,19 +5183,19 @@
         <v>20</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH30" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="AI30" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AJ30" t="s" s="2">
-        <v>101</v>
+        <v>140</v>
       </c>
       <c r="AK30" t="s" s="2">
         <v>20</v>
@@ -5172,7 +5204,7 @@
         <v>20</v>
       </c>
       <c r="AM30" t="s" s="2">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="AN30" t="s" s="2">
         <v>20</v>
@@ -5187,26 +5219,26 @@
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
-        <v>20</v>
+        <v>317</v>
       </c>
       <c r="E31" s="2"/>
       <c r="F31" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="G31" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="H31" t="s" s="2">
         <v>20</v>
       </c>
       <c r="I31" t="s" s="2">
-        <v>20</v>
+        <v>90</v>
       </c>
       <c r="J31" t="s" s="2">
         <v>90</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>317</v>
+        <v>134</v>
       </c>
       <c r="L31" t="s" s="2">
         <v>318</v>
@@ -5214,8 +5246,12 @@
       <c r="M31" t="s" s="2">
         <v>319</v>
       </c>
-      <c r="N31" s="2"/>
-      <c r="O31" s="2"/>
+      <c r="N31" t="s" s="2">
+        <v>151</v>
+      </c>
+      <c r="O31" t="s" s="2">
+        <v>152</v>
+      </c>
       <c r="P31" t="s" s="2">
         <v>20</v>
       </c>
@@ -5263,19 +5299,19 @@
         <v>20</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="AG31" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="AH31" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="AI31" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AJ31" t="s" s="2">
-        <v>101</v>
+        <v>140</v>
       </c>
       <c r="AK31" t="s" s="2">
         <v>20</v>
@@ -5284,7 +5320,7 @@
         <v>20</v>
       </c>
       <c r="AM31" t="s" s="2">
-        <v>320</v>
+        <v>132</v>
       </c>
       <c r="AN31" t="s" s="2">
         <v>20</v>
@@ -5299,7 +5335,7 @@
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
-        <v>322</v>
+        <v>20</v>
       </c>
       <c r="E32" s="2"/>
       <c r="F32" t="s" s="2">
@@ -5318,15 +5354,17 @@
         <v>20</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>296</v>
+        <v>307</v>
       </c>
       <c r="L32" t="s" s="2">
+        <v>322</v>
+      </c>
+      <c r="M32" t="s" s="2">
         <v>323</v>
       </c>
-      <c r="M32" t="s" s="2">
+      <c r="N32" t="s" s="2">
         <v>324</v>
       </c>
-      <c r="N32" s="2"/>
       <c r="O32" t="s" s="2">
         <v>325</v>
       </c>
@@ -5395,10 +5433,10 @@
         <v>20</v>
       </c>
       <c r="AL32" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AM32" t="s" s="2">
         <v>326</v>
-      </c>
-      <c r="AM32" t="s" s="2">
-        <v>327</v>
       </c>
       <c r="AN32" t="s" s="2">
         <v>20</v>
@@ -5406,10 +5444,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -5417,10 +5455,10 @@
       </c>
       <c r="E33" s="2"/>
       <c r="F33" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="G33" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="H33" t="s" s="2">
         <v>20</v>
@@ -5429,10 +5467,10 @@
         <v>20</v>
       </c>
       <c r="J33" t="s" s="2">
-        <v>20</v>
+        <v>90</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>187</v>
+        <v>328</v>
       </c>
       <c r="L33" t="s" s="2">
         <v>329</v>
@@ -5465,13 +5503,13 @@
         <v>20</v>
       </c>
       <c r="X33" t="s" s="2">
-        <v>191</v>
+        <v>20</v>
       </c>
       <c r="Y33" t="s" s="2">
-        <v>331</v>
+        <v>20</v>
       </c>
       <c r="Z33" t="s" s="2">
-        <v>332</v>
+        <v>20</v>
       </c>
       <c r="AA33" t="s" s="2">
         <v>20</v>
@@ -5489,13 +5527,13 @@
         <v>20</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="AG33" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="AH33" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="AI33" t="s" s="2">
         <v>20</v>
@@ -5507,10 +5545,10 @@
         <v>20</v>
       </c>
       <c r="AL33" t="s" s="2">
-        <v>326</v>
+        <v>20</v>
       </c>
       <c r="AM33" t="s" s="2">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="AN33" t="s" s="2">
         <v>20</v>
@@ -5518,21 +5556,21 @@
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
-        <v>20</v>
+        <v>333</v>
       </c>
       <c r="E34" s="2"/>
       <c r="F34" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G34" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="H34" t="s" s="2">
         <v>20</v>
@@ -5544,19 +5582,17 @@
         <v>20</v>
       </c>
       <c r="K34" t="s" s="2">
+        <v>307</v>
+      </c>
+      <c r="L34" t="s" s="2">
+        <v>334</v>
+      </c>
+      <c r="M34" t="s" s="2">
         <v>335</v>
       </c>
-      <c r="L34" t="s" s="2">
+      <c r="N34" s="2"/>
+      <c r="O34" t="s" s="2">
         <v>336</v>
-      </c>
-      <c r="M34" t="s" s="2">
-        <v>337</v>
-      </c>
-      <c r="N34" t="s" s="2">
-        <v>338</v>
-      </c>
-      <c r="O34" t="s" s="2">
-        <v>339</v>
       </c>
       <c r="P34" t="s" s="2">
         <v>20</v>
@@ -5593,23 +5629,25 @@
         <v>20</v>
       </c>
       <c r="AB34" t="s" s="2">
-        <v>340</v>
-      </c>
-      <c r="AC34" s="2"/>
+        <v>20</v>
+      </c>
+      <c r="AC34" t="s" s="2">
+        <v>20</v>
+      </c>
       <c r="AD34" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AE34" t="s" s="2">
-        <v>138</v>
+        <v>20</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH34" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="AI34" t="s" s="2">
         <v>20</v>
@@ -5621,10 +5659,10 @@
         <v>20</v>
       </c>
       <c r="AL34" t="s" s="2">
-        <v>326</v>
+        <v>337</v>
       </c>
       <c r="AM34" t="s" s="2">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="AN34" t="s" s="2">
         <v>20</v>
@@ -5632,14 +5670,12 @@
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>334</v>
-      </c>
-      <c r="C35" t="s" s="2">
-        <v>343</v>
-      </c>
+        <v>339</v>
+      </c>
+      <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
         <v>20</v>
       </c>
@@ -5660,20 +5696,16 @@
         <v>20</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>344</v>
+        <v>187</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>337</v>
-      </c>
-      <c r="N35" t="s" s="2">
-        <v>338</v>
-      </c>
-      <c r="O35" t="s" s="2">
-        <v>339</v>
-      </c>
+        <v>341</v>
+      </c>
+      <c r="N35" s="2"/>
+      <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
         <v>20</v>
       </c>
@@ -5697,13 +5729,13 @@
         <v>20</v>
       </c>
       <c r="X35" t="s" s="2">
-        <v>20</v>
+        <v>191</v>
       </c>
       <c r="Y35" t="s" s="2">
-        <v>20</v>
+        <v>342</v>
       </c>
       <c r="Z35" t="s" s="2">
-        <v>20</v>
+        <v>343</v>
       </c>
       <c r="AA35" t="s" s="2">
         <v>20</v>
@@ -5721,7 +5753,7 @@
         <v>20</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>78</v>
@@ -5739,10 +5771,10 @@
         <v>20</v>
       </c>
       <c r="AL35" t="s" s="2">
-        <v>326</v>
+        <v>337</v>
       </c>
       <c r="AM35" t="s" s="2">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="AN35" t="s" s="2">
         <v>20</v>
@@ -5753,11 +5785,9 @@
         <v>345</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>334</v>
-      </c>
-      <c r="C36" t="s" s="2">
-        <v>346</v>
-      </c>
+        <v>345</v>
+      </c>
+      <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
         <v>20</v>
       </c>
@@ -5778,19 +5808,19 @@
         <v>20</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="L36" t="s" s="2">
         <v>347</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>337</v>
+        <v>348</v>
       </c>
       <c r="N36" t="s" s="2">
-        <v>338</v>
+        <v>349</v>
       </c>
       <c r="O36" t="s" s="2">
-        <v>339</v>
+        <v>350</v>
       </c>
       <c r="P36" t="s" s="2">
         <v>20</v>
@@ -5827,19 +5857,17 @@
         <v>20</v>
       </c>
       <c r="AB36" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AC36" t="s" s="2">
-        <v>20</v>
-      </c>
+        <v>351</v>
+      </c>
+      <c r="AC36" s="2"/>
       <c r="AD36" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AE36" t="s" s="2">
-        <v>20</v>
+        <v>138</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>334</v>
+        <v>345</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>78</v>
@@ -5857,10 +5885,10 @@
         <v>20</v>
       </c>
       <c r="AL36" t="s" s="2">
-        <v>326</v>
+        <v>337</v>
       </c>
       <c r="AM36" t="s" s="2">
-        <v>341</v>
+        <v>352</v>
       </c>
       <c r="AN36" t="s" s="2">
         <v>20</v>
@@ -5868,12 +5896,14 @@
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>349</v>
-      </c>
-      <c r="C37" s="2"/>
+        <v>345</v>
+      </c>
+      <c r="C37" t="s" s="2">
+        <v>354</v>
+      </c>
       <c r="D37" t="s" s="2">
         <v>20</v>
       </c>
@@ -5882,7 +5912,7 @@
         <v>78</v>
       </c>
       <c r="G37" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="H37" t="s" s="2">
         <v>20</v>
@@ -5894,16 +5924,20 @@
         <v>20</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>296</v>
+        <v>355</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>297</v>
+        <v>347</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>298</v>
-      </c>
-      <c r="N37" s="2"/>
-      <c r="O37" s="2"/>
+        <v>348</v>
+      </c>
+      <c r="N37" t="s" s="2">
+        <v>349</v>
+      </c>
+      <c r="O37" t="s" s="2">
+        <v>350</v>
+      </c>
       <c r="P37" t="s" s="2">
         <v>20</v>
       </c>
@@ -5951,28 +5985,28 @@
         <v>20</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>299</v>
+        <v>345</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH37" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="AI37" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AJ37" t="s" s="2">
-        <v>20</v>
+        <v>101</v>
       </c>
       <c r="AK37" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL37" t="s" s="2">
-        <v>20</v>
+        <v>337</v>
       </c>
       <c r="AM37" t="s" s="2">
-        <v>300</v>
+        <v>352</v>
       </c>
       <c r="AN37" t="s" s="2">
         <v>20</v>
@@ -5980,14 +6014,16 @@
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>350</v>
+        <v>356</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>351</v>
-      </c>
-      <c r="C38" s="2"/>
+        <v>345</v>
+      </c>
+      <c r="C38" t="s" s="2">
+        <v>357</v>
+      </c>
       <c r="D38" t="s" s="2">
-        <v>148</v>
+        <v>20</v>
       </c>
       <c r="E38" s="2"/>
       <c r="F38" t="s" s="2">
@@ -6006,18 +6042,20 @@
         <v>20</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>134</v>
+        <v>355</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>302</v>
+        <v>358</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>303</v>
+        <v>348</v>
       </c>
       <c r="N38" t="s" s="2">
-        <v>151</v>
-      </c>
-      <c r="O38" s="2"/>
+        <v>349</v>
+      </c>
+      <c r="O38" t="s" s="2">
+        <v>350</v>
+      </c>
       <c r="P38" t="s" s="2">
         <v>20</v>
       </c>
@@ -6053,19 +6091,19 @@
         <v>20</v>
       </c>
       <c r="AB38" t="s" s="2">
-        <v>137</v>
+        <v>20</v>
       </c>
       <c r="AC38" t="s" s="2">
-        <v>352</v>
+        <v>20</v>
       </c>
       <c r="AD38" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AE38" t="s" s="2">
-        <v>138</v>
+        <v>20</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>304</v>
+        <v>345</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>78</v>
@@ -6077,16 +6115,16 @@
         <v>20</v>
       </c>
       <c r="AJ38" t="s" s="2">
-        <v>140</v>
+        <v>101</v>
       </c>
       <c r="AK38" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL38" t="s" s="2">
-        <v>20</v>
+        <v>337</v>
       </c>
       <c r="AM38" t="s" s="2">
-        <v>300</v>
+        <v>352</v>
       </c>
       <c r="AN38" t="s" s="2">
         <v>20</v>
@@ -6094,14 +6132,12 @@
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>353</v>
+        <v>359</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>351</v>
-      </c>
-      <c r="C39" t="s" s="2">
-        <v>354</v>
-      </c>
+        <v>360</v>
+      </c>
+      <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
         <v>20</v>
       </c>
@@ -6110,7 +6146,7 @@
         <v>78</v>
       </c>
       <c r="G39" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="H39" t="s" s="2">
         <v>20</v>
@@ -6122,13 +6158,13 @@
         <v>20</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>355</v>
+        <v>307</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>356</v>
+        <v>308</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>357</v>
+        <v>309</v>
       </c>
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
@@ -6179,19 +6215,19 @@
         <v>20</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH39" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="AI39" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AJ39" t="s" s="2">
-        <v>140</v>
+        <v>20</v>
       </c>
       <c r="AK39" t="s" s="2">
         <v>20</v>
@@ -6200,7 +6236,7 @@
         <v>20</v>
       </c>
       <c r="AM39" t="s" s="2">
-        <v>20</v>
+        <v>311</v>
       </c>
       <c r="AN39" t="s" s="2">
         <v>20</v>
@@ -6208,23 +6244,21 @@
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>351</v>
-      </c>
-      <c r="C40" t="s" s="2">
-        <v>359</v>
-      </c>
+        <v>362</v>
+      </c>
+      <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
-        <v>20</v>
+        <v>148</v>
       </c>
       <c r="E40" s="2"/>
       <c r="F40" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G40" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="H40" t="s" s="2">
         <v>20</v>
@@ -6236,15 +6270,17 @@
         <v>20</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>360</v>
+        <v>134</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>361</v>
+        <v>313</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>362</v>
-      </c>
-      <c r="N40" s="2"/>
+        <v>314</v>
+      </c>
+      <c r="N40" t="s" s="2">
+        <v>151</v>
+      </c>
       <c r="O40" s="2"/>
       <c r="P40" t="s" s="2">
         <v>20</v>
@@ -6281,19 +6317,19 @@
         <v>20</v>
       </c>
       <c r="AB40" t="s" s="2">
-        <v>20</v>
+        <v>137</v>
       </c>
       <c r="AC40" t="s" s="2">
-        <v>20</v>
+        <v>363</v>
       </c>
       <c r="AD40" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AE40" t="s" s="2">
-        <v>20</v>
+        <v>138</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>304</v>
+        <v>315</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>78</v>
@@ -6314,7 +6350,7 @@
         <v>20</v>
       </c>
       <c r="AM40" t="s" s="2">
-        <v>20</v>
+        <v>311</v>
       </c>
       <c r="AN40" t="s" s="2">
         <v>20</v>
@@ -6322,12 +6358,14 @@
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>364</v>
-      </c>
-      <c r="C41" s="2"/>
+        <v>362</v>
+      </c>
+      <c r="C41" t="s" s="2">
+        <v>365</v>
+      </c>
       <c r="D41" t="s" s="2">
         <v>20</v>
       </c>
@@ -6336,7 +6374,7 @@
         <v>78</v>
       </c>
       <c r="G41" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="H41" t="s" s="2">
         <v>20</v>
@@ -6345,21 +6383,19 @@
         <v>20</v>
       </c>
       <c r="J41" t="s" s="2">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>109</v>
+        <v>366</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="N41" s="2"/>
-      <c r="O41" t="s" s="2">
-        <v>367</v>
-      </c>
+      <c r="O41" s="2"/>
       <c r="P41" t="s" s="2">
         <v>20</v>
       </c>
@@ -6371,7 +6407,7 @@
         <v>20</v>
       </c>
       <c r="T41" t="s" s="2">
-        <v>368</v>
+        <v>20</v>
       </c>
       <c r="U41" t="s" s="2">
         <v>20</v>
@@ -6383,13 +6419,13 @@
         <v>20</v>
       </c>
       <c r="X41" t="s" s="2">
-        <v>179</v>
+        <v>20</v>
       </c>
       <c r="Y41" t="s" s="2">
-        <v>369</v>
+        <v>20</v>
       </c>
       <c r="Z41" t="s" s="2">
-        <v>370</v>
+        <v>20</v>
       </c>
       <c r="AA41" t="s" s="2">
         <v>20</v>
@@ -6407,28 +6443,28 @@
         <v>20</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>371</v>
+        <v>315</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH41" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="AI41" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AJ41" t="s" s="2">
-        <v>101</v>
+        <v>140</v>
       </c>
       <c r="AK41" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL41" t="s" s="2">
-        <v>372</v>
+        <v>20</v>
       </c>
       <c r="AM41" t="s" s="2">
-        <v>373</v>
+        <v>20</v>
       </c>
       <c r="AN41" t="s" s="2">
         <v>20</v>
@@ -6436,12 +6472,14 @@
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>375</v>
-      </c>
-      <c r="C42" s="2"/>
+        <v>362</v>
+      </c>
+      <c r="C42" t="s" s="2">
+        <v>370</v>
+      </c>
       <c r="D42" t="s" s="2">
         <v>20</v>
       </c>
@@ -6459,21 +6497,19 @@
         <v>20</v>
       </c>
       <c r="J42" t="s" s="2">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>109</v>
+        <v>371</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="N42" s="2"/>
-      <c r="O42" t="s" s="2">
-        <v>378</v>
-      </c>
+      <c r="O42" s="2"/>
       <c r="P42" t="s" s="2">
         <v>20</v>
       </c>
@@ -6485,7 +6521,7 @@
         <v>20</v>
       </c>
       <c r="T42" t="s" s="2">
-        <v>379</v>
+        <v>20</v>
       </c>
       <c r="U42" t="s" s="2">
         <v>20</v>
@@ -6497,13 +6533,13 @@
         <v>20</v>
       </c>
       <c r="X42" t="s" s="2">
-        <v>113</v>
+        <v>20</v>
       </c>
       <c r="Y42" t="s" s="2">
-        <v>114</v>
+        <v>20</v>
       </c>
       <c r="Z42" t="s" s="2">
-        <v>115</v>
+        <v>20</v>
       </c>
       <c r="AA42" t="s" s="2">
         <v>20</v>
@@ -6521,19 +6557,19 @@
         <v>20</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>380</v>
+        <v>315</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH42" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="AI42" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AJ42" t="s" s="2">
-        <v>101</v>
+        <v>140</v>
       </c>
       <c r="AK42" t="s" s="2">
         <v>20</v>
@@ -6542,7 +6578,7 @@
         <v>20</v>
       </c>
       <c r="AM42" t="s" s="2">
-        <v>381</v>
+        <v>20</v>
       </c>
       <c r="AN42" t="s" s="2">
         <v>20</v>
@@ -6550,10 +6586,10 @@
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>382</v>
+        <v>374</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>383</v>
+        <v>375</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -6564,7 +6600,7 @@
         <v>78</v>
       </c>
       <c r="G43" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="H43" t="s" s="2">
         <v>20</v>
@@ -6573,22 +6609,20 @@
         <v>20</v>
       </c>
       <c r="J43" t="s" s="2">
-        <v>20</v>
+        <v>90</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>384</v>
+        <v>109</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>385</v>
+        <v>376</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>386</v>
-      </c>
-      <c r="N43" t="s" s="2">
-        <v>387</v>
-      </c>
+        <v>377</v>
+      </c>
+      <c r="N43" s="2"/>
       <c r="O43" t="s" s="2">
-        <v>388</v>
+        <v>378</v>
       </c>
       <c r="P43" t="s" s="2">
         <v>20</v>
@@ -6601,7 +6635,7 @@
         <v>20</v>
       </c>
       <c r="T43" t="s" s="2">
-        <v>20</v>
+        <v>379</v>
       </c>
       <c r="U43" t="s" s="2">
         <v>20</v>
@@ -6613,13 +6647,13 @@
         <v>20</v>
       </c>
       <c r="X43" t="s" s="2">
-        <v>20</v>
+        <v>179</v>
       </c>
       <c r="Y43" t="s" s="2">
-        <v>20</v>
+        <v>380</v>
       </c>
       <c r="Z43" t="s" s="2">
-        <v>20</v>
+        <v>381</v>
       </c>
       <c r="AA43" t="s" s="2">
         <v>20</v>
@@ -6637,7 +6671,7 @@
         <v>20</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>389</v>
+        <v>382</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>78</v>
@@ -6655,10 +6689,10 @@
         <v>20</v>
       </c>
       <c r="AL43" t="s" s="2">
-        <v>390</v>
+        <v>383</v>
       </c>
       <c r="AM43" t="s" s="2">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="AN43" t="s" s="2">
         <v>20</v>
@@ -6666,10 +6700,10 @@
     </row>
     <row r="44">
       <c r="A44" t="s" s="2">
-        <v>392</v>
+        <v>385</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>393</v>
+        <v>386</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -6677,7 +6711,7 @@
       </c>
       <c r="E44" s="2"/>
       <c r="F44" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="G44" t="s" s="2">
         <v>89</v>
@@ -6692,19 +6726,17 @@
         <v>90</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>394</v>
+        <v>109</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>395</v>
+        <v>387</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>396</v>
-      </c>
-      <c r="N44" t="s" s="2">
-        <v>397</v>
-      </c>
+        <v>388</v>
+      </c>
+      <c r="N44" s="2"/>
       <c r="O44" t="s" s="2">
-        <v>398</v>
+        <v>389</v>
       </c>
       <c r="P44" t="s" s="2">
         <v>20</v>
@@ -6717,7 +6749,7 @@
         <v>20</v>
       </c>
       <c r="T44" t="s" s="2">
-        <v>399</v>
+        <v>390</v>
       </c>
       <c r="U44" t="s" s="2">
         <v>20</v>
@@ -6729,13 +6761,13 @@
         <v>20</v>
       </c>
       <c r="X44" t="s" s="2">
-        <v>20</v>
+        <v>113</v>
       </c>
       <c r="Y44" t="s" s="2">
-        <v>20</v>
+        <v>114</v>
       </c>
       <c r="Z44" t="s" s="2">
-        <v>20</v>
+        <v>115</v>
       </c>
       <c r="AA44" t="s" s="2">
         <v>20</v>
@@ -6753,7 +6785,7 @@
         <v>20</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>400</v>
+        <v>391</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>78</v>
@@ -6771,10 +6803,10 @@
         <v>20</v>
       </c>
       <c r="AL44" t="s" s="2">
-        <v>401</v>
+        <v>20</v>
       </c>
       <c r="AM44" t="s" s="2">
-        <v>402</v>
+        <v>392</v>
       </c>
       <c r="AN44" t="s" s="2">
         <v>20</v>
@@ -6782,10 +6814,10 @@
     </row>
     <row r="45">
       <c r="A45" t="s" s="2">
-        <v>403</v>
+        <v>393</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>404</v>
+        <v>394</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -6796,7 +6828,7 @@
         <v>78</v>
       </c>
       <c r="G45" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="H45" t="s" s="2">
         <v>20</v>
@@ -6805,22 +6837,22 @@
         <v>20</v>
       </c>
       <c r="J45" t="s" s="2">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>405</v>
+        <v>395</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>406</v>
+        <v>396</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>407</v>
+        <v>397</v>
       </c>
       <c r="N45" t="s" s="2">
-        <v>408</v>
+        <v>398</v>
       </c>
       <c r="O45" t="s" s="2">
-        <v>409</v>
+        <v>399</v>
       </c>
       <c r="P45" t="s" s="2">
         <v>20</v>
@@ -6869,7 +6901,7 @@
         <v>20</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>410</v>
+        <v>400</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>78</v>
@@ -6887,10 +6919,10 @@
         <v>20</v>
       </c>
       <c r="AL45" t="s" s="2">
-        <v>20</v>
+        <v>401</v>
       </c>
       <c r="AM45" t="s" s="2">
-        <v>411</v>
+        <v>402</v>
       </c>
       <c r="AN45" t="s" s="2">
         <v>20</v>
@@ -6898,10 +6930,10 @@
     </row>
     <row r="46">
       <c r="A46" t="s" s="2">
-        <v>412</v>
+        <v>403</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>413</v>
+        <v>404</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -6909,7 +6941,7 @@
       </c>
       <c r="E46" s="2"/>
       <c r="F46" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="G46" t="s" s="2">
         <v>89</v>
@@ -6924,19 +6956,19 @@
         <v>90</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>384</v>
+        <v>405</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>414</v>
+        <v>406</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>415</v>
+        <v>407</v>
       </c>
       <c r="N46" t="s" s="2">
-        <v>416</v>
+        <v>408</v>
       </c>
       <c r="O46" t="s" s="2">
-        <v>417</v>
+        <v>409</v>
       </c>
       <c r="P46" t="s" s="2">
         <v>20</v>
@@ -6949,7 +6981,7 @@
         <v>20</v>
       </c>
       <c r="T46" t="s" s="2">
-        <v>20</v>
+        <v>410</v>
       </c>
       <c r="U46" t="s" s="2">
         <v>20</v>
@@ -6985,7 +7017,7 @@
         <v>20</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>418</v>
+        <v>411</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>78</v>
@@ -7003,10 +7035,10 @@
         <v>20</v>
       </c>
       <c r="AL46" t="s" s="2">
-        <v>20</v>
+        <v>412</v>
       </c>
       <c r="AM46" t="s" s="2">
-        <v>419</v>
+        <v>413</v>
       </c>
       <c r="AN46" t="s" s="2">
         <v>20</v>
@@ -7014,10 +7046,10 @@
     </row>
     <row r="47">
       <c r="A47" t="s" s="2">
-        <v>420</v>
+        <v>414</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>421</v>
+        <v>415</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -7025,7 +7057,7 @@
       </c>
       <c r="E47" s="2"/>
       <c r="F47" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="G47" t="s" s="2">
         <v>89</v>
@@ -7040,17 +7072,19 @@
         <v>90</v>
       </c>
       <c r="K47" t="s" s="2">
-        <v>296</v>
+        <v>416</v>
       </c>
       <c r="L47" t="s" s="2">
-        <v>422</v>
+        <v>417</v>
       </c>
       <c r="M47" t="s" s="2">
-        <v>423</v>
-      </c>
-      <c r="N47" s="2"/>
+        <v>418</v>
+      </c>
+      <c r="N47" t="s" s="2">
+        <v>419</v>
+      </c>
       <c r="O47" t="s" s="2">
-        <v>424</v>
+        <v>420</v>
       </c>
       <c r="P47" t="s" s="2">
         <v>20</v>
@@ -7060,10 +7094,10 @@
         <v>20</v>
       </c>
       <c r="S47" t="s" s="2">
-        <v>425</v>
+        <v>20</v>
       </c>
       <c r="T47" t="s" s="2">
-        <v>426</v>
+        <v>20</v>
       </c>
       <c r="U47" t="s" s="2">
         <v>20</v>
@@ -7099,7 +7133,7 @@
         <v>20</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>427</v>
+        <v>421</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>78</v>
@@ -7120,7 +7154,7 @@
         <v>20</v>
       </c>
       <c r="AM47" t="s" s="2">
-        <v>428</v>
+        <v>422</v>
       </c>
       <c r="AN47" t="s" s="2">
         <v>20</v>
@@ -7128,10 +7162,10 @@
     </row>
     <row r="48">
       <c r="A48" t="s" s="2">
-        <v>429</v>
+        <v>423</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -7154,17 +7188,19 @@
         <v>90</v>
       </c>
       <c r="K48" t="s" s="2">
-        <v>431</v>
+        <v>395</v>
       </c>
       <c r="L48" t="s" s="2">
-        <v>432</v>
+        <v>425</v>
       </c>
       <c r="M48" t="s" s="2">
-        <v>433</v>
-      </c>
-      <c r="N48" s="2"/>
+        <v>426</v>
+      </c>
+      <c r="N48" t="s" s="2">
+        <v>427</v>
+      </c>
       <c r="O48" t="s" s="2">
-        <v>434</v>
+        <v>428</v>
       </c>
       <c r="P48" t="s" s="2">
         <v>20</v>
@@ -7213,7 +7249,7 @@
         <v>20</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>435</v>
+        <v>429</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>78</v>
@@ -7234,9 +7270,237 @@
         <v>20</v>
       </c>
       <c r="AM48" t="s" s="2">
-        <v>411</v>
+        <v>430</v>
       </c>
       <c r="AN48" t="s" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s" s="2">
+        <v>431</v>
+      </c>
+      <c r="B49" t="s" s="2">
+        <v>432</v>
+      </c>
+      <c r="C49" s="2"/>
+      <c r="D49" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="E49" s="2"/>
+      <c r="F49" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="G49" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="H49" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="I49" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="J49" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="K49" t="s" s="2">
+        <v>307</v>
+      </c>
+      <c r="L49" t="s" s="2">
+        <v>433</v>
+      </c>
+      <c r="M49" t="s" s="2">
+        <v>434</v>
+      </c>
+      <c r="N49" s="2"/>
+      <c r="O49" t="s" s="2">
+        <v>435</v>
+      </c>
+      <c r="P49" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="Q49" s="2"/>
+      <c r="R49" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="S49" t="s" s="2">
+        <v>436</v>
+      </c>
+      <c r="T49" t="s" s="2">
+        <v>437</v>
+      </c>
+      <c r="U49" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="V49" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="W49" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="X49" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="Y49" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="Z49" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AA49" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AB49" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AC49" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AD49" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AE49" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AF49" t="s" s="2">
+        <v>438</v>
+      </c>
+      <c r="AG49" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH49" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AI49" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AJ49" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="AK49" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AL49" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AM49" t="s" s="2">
+        <v>439</v>
+      </c>
+      <c r="AN49" t="s" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s" s="2">
+        <v>440</v>
+      </c>
+      <c r="B50" t="s" s="2">
+        <v>441</v>
+      </c>
+      <c r="C50" s="2"/>
+      <c r="D50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="E50" s="2"/>
+      <c r="F50" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G50" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="H50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="I50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="J50" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="K50" t="s" s="2">
+        <v>442</v>
+      </c>
+      <c r="L50" t="s" s="2">
+        <v>443</v>
+      </c>
+      <c r="M50" t="s" s="2">
+        <v>444</v>
+      </c>
+      <c r="N50" s="2"/>
+      <c r="O50" t="s" s="2">
+        <v>445</v>
+      </c>
+      <c r="P50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="Q50" s="2"/>
+      <c r="R50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="S50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="T50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="U50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="V50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="W50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="X50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="Y50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="Z50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AA50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AB50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AC50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AD50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AE50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AF50" t="s" s="2">
+        <v>446</v>
+      </c>
+      <c r="AG50" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH50" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AI50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AJ50" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="AK50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AL50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AM50" t="s" s="2">
+        <v>422</v>
+      </c>
+      <c r="AN50" t="s" s="2">
         <v>20</v>
       </c>
     </row>

</xml_diff>